<commit_message>
feat(review): add themeable cross-format comment UI
Add a built-in read-only comment presentation for DOCX, PPTX, and XLSX while preserving primitive data and geometry APIs for application-owned interfaces. Keep card structure stable and CSS-themeable, remeasure geometry changes independently of optional connectors, and expose comment-aware selection context across formats.

Restore the public documentation boundary: format pages contain live examples, API tables live under /api, and shared ownership, rendering-mode, and optional-renderer guidance lives under /production. Add format comment demos and focused architecture, API, layout, and theme coverage.

Verification: focused comment/API/site tests (269 passed); full site tests (159 passed); Astro static build (31 pages); viewer API symmetry check; git diff --check.

Co-Authored-By: Codex GPT-5 <noreply@openai.com>
</commit_message>
<xml_diff>
--- a/packages/xlsx/public/demo/sample-1.xlsx
+++ b/packages/xlsx/public/demo/sample-1.xlsx
@@ -37,6 +37,23 @@
     </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac">
+  <authors>
+    <author>tc={11111111-1111-4111-8111-111111111111}</author>
+  </authors>
+  <commentList>
+    <comment ref="B18" authorId="0" x15ac:uid="{11111111-1111-4111-8111-111111111111}">
+      <text>
+        <t>[Threaded comment]
+Confirm this regional summary before publishing.
+Reply: Verified against the source inventory.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5390,6 +5407,12 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
+  <xltc:person displayName="Olivia Bennett" id="{33333333-3333-4333-8333-333333333333}"/>
+</xltc:personList>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office テーマ">
   <a:themeElements>
@@ -5705,6 +5728,17 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedcomments/threadedcomment.xml><?xml version="1.0" encoding="utf-8"?>
+<xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
+  <xltc:threadedComment ref="B18" dT="2026-08-25T13:00:00Z" personId="{33333333-3333-4333-8333-333333333333}" id="{11111111-1111-4111-8111-111111111111}">
+    <xltc:text>Confirm this regional summary before publishing.</xltc:text>
+  </xltc:threadedComment>
+  <xltc:threadedComment ref="B18" dT="2026-08-25T13:01:00Z" personId="{33333333-3333-4333-8333-333333333333}" id="{22222222-2222-4222-8222-222222222222}" parentId="{11111111-1111-4111-8111-111111111111}">
+    <xltc:text>Verified against the source inventory.</xltc:text>
+  </xltc:threadedComment>
+</xltc:ThreadedComments>
+</file>
+
 <file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
 <wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
   <wetp:taskpane dockstate="right" visibility="0" width="350" row="0">
@@ -6339,6 +6373,7 @@
         <cfvo type="max"/>
         <color rgb="FF95D5B2"/>
       </dataBar>
+      <legacyDrawing r:id="rIdCommentVml"/>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
           <x14:id>{190A5F63-8D89-A941-BDCE-58ACFB08F9A9}</x14:id>

</xml_diff>